<commit_message>
Updated to include rationale from data standards manual
</commit_message>
<xml_diff>
--- a/Foundation Layer/Ontology Generator/datasource/DataDictionaryAnnotations.xlsx
+++ b/Foundation Layer/Ontology Generator/datasource/DataDictionaryAnnotations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\61084\Desktop\NHDAP Data Lab\ICF Data Lab\GT.Data.Exchange.and.Interoperability\Foundation Layer\Ontology Generator\datasource\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8461A30E-0158-4948-8ABF-A68C222A04C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F03E51E-C9D4-447A-B71A-C0DD2C6A35D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data Elements" sheetId="1" r:id="rId1"/>
@@ -172,7 +172,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="792" uniqueCount="391">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="949" uniqueCount="544">
   <si>
     <t>Element Identifier</t>
   </si>
@@ -1345,13 +1345,582 @@
   </si>
   <si>
     <t>Export</t>
+  </si>
+  <si>
+    <t>Rationale</t>
+  </si>
+  <si>
+    <t>Data Collection Instruction</t>
+  </si>
+  <si>
+    <t>To uniquely identify organizations operating one or more projects that enter data into HMIS, as well as any organizations operating residential continuum projects that are not participating in HMIS. This element is also used to identify organizations that are classified as Victim Service Providers (VSPs).</t>
+  </si>
+  <si>
+    <t>To identify each project entering data into HMIS, as well as any residential continuum projects not participating in HMIS; and to associate each project with the specific type of lodging or services provided and the details about those project types. The 'Project ID' is used to link project descriptor information in other data elements to the specific project, and to link clients and their enrollment data to the project. Data related to project type is necessary to identify corresponding data collection requirements and for reporting purposes. The element also identifies whether the project is a continuum project, Rapid Re-Housing subtypes, and the relationship of a 'Services Only' project (or RRH: Services Only subtype) to a housing project as necessary. Finally, HOPWA-funded projects identify whether they are 'Medically Assisted Living Facilities' at this stage of project setup.</t>
+  </si>
+  <si>
+    <t>To associate each project entering data into HMIS, as well as any residential continuum projects not participating in HMIS, with one or more Continuum of Care (CoC) for reporting and data exchange purposes.</t>
+  </si>
+  <si>
+    <t>To identify funding sources for each project entering data into HMIS, as well as any residential continuum projects not participating in HMIS, and associate projects with corresponding data collection requirements and reporting specifications.</t>
+  </si>
+  <si>
+    <t>To record bed and unit inventory information for each residential project entering data into HMIS, as well as any residential continuum projects not participating in HMIS, for use in tracking utilization, data quality analysis, and reporting.</t>
+  </si>
+  <si>
+    <t>To identify the HMIS or comparable database participation status of all Continuum projects.</t>
+  </si>
+  <si>
+    <r>
+      <t>The </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF333333"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Coordinated Entry Participation Status</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF333333"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> is designed to identify a project’s type of engagement in the local Coordinated Entry System (CES). This element captures information about whether a project is an access point for the CES and if the project accepts referrals </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF333333"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>from</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF333333"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> the CES.</t>
+    </r>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/project-descriptor-data-elements/209-coordinated-entry-participation-status/</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/project-descriptor-data-elements/208-hmis-participation-status/</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/project-descriptor-data-elements/207-bed-and-unit-inventory-information/</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/project-descriptor-data-elements/206-funding-sources/</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/project-descriptor-data-elements/203-continuum-of-care-information/</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/project-descriptor-data-elements/202-project-information/</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/project-descriptor-data-elements/201-organization-information/</t>
+  </si>
+  <si>
+    <t>To support the unique identification of each person served.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/universal-data-elements/301-name/</t>
+  </si>
+  <si>
+    <t>To support the unique identification of each person served.
+Where data is shared across projects, the Social Security Number (SSN) greatly facilitates the process of identifying clients who have been served and allows projects to avoid creating duplicate records at Project Start.
+Where data is not shared, CoCs rely on unique identifiers to produce an unduplicated count in the HMIS. Name and date of birth are useful unique identifiers, but the SSN is helpful for deduplicating clients where name and/or date of birth might be the same.
+Also, an important objective for ending homelessness is to increase access and utilization of mainstream programs by persons who are experiencing homelessness or are at-risk of homelessness. Since SSN is a required data element for many mainstream programs, projects may need the SSN to help their clients access mainstream services.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/universal-data-elements/302-social-security-number/</t>
+  </si>
+  <si>
+    <t>To calculate the age of persons served at the time of project start or at any point during project enrollment and to support the unique identification of each person served.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/universal-data-elements/303-date-of-birth/</t>
+  </si>
+  <si>
+    <r>
+      <t>To indicate client’s </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF333333"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>self-identification</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF333333"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> with one or more different racial and/or ethnic categories. This data supports system planning, and local and national understanding of who is experiencing homelessness.</t>
+    </r>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/universal-data-elements/304-race-and-ethnicity/</t>
+  </si>
+  <si>
+    <t>To indicate whether clients have ever spent time in the United States Armed Forces and may be eligible for VA Homeless Programs. Allows for an accurate count of how many Veterans experience homelessness. Useful for screening for possible housing and service interventions and for gaining understanding of Veterans' service needs.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/universal-data-elements/307-veteran-status/</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/universal-data-elements/308-disabling-condition/</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/universal-data-elements/316-enrollment-coc/</t>
+  </si>
+  <si>
+    <t>To indicate whether clients have a disabling condition as defined below. This data element is to be used with other information to identify whether a client meets the criteria for experiencing chronic homelessness.</t>
+  </si>
+  <si>
+    <r>
+      <t>To determine the start of each client's period of participation with a project. All projects need this data element for reporting time spent participating in the project by a given client. Paired with </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF333333"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>3.20 ‘Housing Move-In Date’</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF333333"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>, it becomes possible to determine the length of time from project start to housing placement for all clients accessing permanent housing.</t>
+    </r>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/universal-data-elements/310-project-start-date/</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/universal-data-elements/311-project-exit-date/</t>
+  </si>
+  <si>
+    <t>To determine the end of a client's period of participation with a project. All projects need this data element for reporting time spent participating in the project.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/universal-data-elements/312-destination/</t>
+  </si>
+  <si>
+    <t>To identify where a client will stay just after exiting a project for purposes of tracking and outcome measurement.</t>
+  </si>
+  <si>
+    <t>To identify one person to whom all other household members can be linked to at the time they enter a project. This facilitates the identification and enumeration of households. In addition, specifying the relationship of household members to the Head of Household facilitates reporting on household composition.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/universal-data-elements/315-relationship-to-head-of-household/</t>
+  </si>
+  <si>
+    <t>To link client household data to the relevant CoC in which the assisting project operates. Necessary for projects that operate across multiple CoCs for data export purposes and to ensure accurate counts of persons who are served within a CoC. </t>
+  </si>
+  <si>
+    <t>To document the date that a household moves into housing. This date differentiates households that have already moved into permanent housing from households that are still experiencing literal homelessness (in Emergency Shelter, Safe Haven, Transitional Housing, or on the street) as they prepare to move into an available unit. This is critical to Housing Inventory Count (HIC) and Point-in-Time (PIT) counts.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/universal-data-elements/320-housing-move-in-date/</t>
+  </si>
+  <si>
+    <t>To identify the type of living situation and length of stay in that situation immediately prior to project start for all adults and the Head of Household. This data element is used with other information to identify whether a client appears to meet the criteria for experiencing chronic homelessness at various points of enrollment (i.e., at the point of project entry, at a point during a project enrollment, or at any point over the course of a specified reporting period).</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/universal-data-elements/3917-prior-living-situation/</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/common-program-specific-data-elements/421-sex/</t>
+  </si>
+  <si>
+    <t>To create separate counts of females and males experiencing homelessness.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/common-program-specific-data-elements/420-coordinated-entry-event/</t>
+  </si>
+  <si>
+    <t>The Coordinated Entry Event element is designed to capture key referral and placement events, as well as the results of those events. It will help communities understand the events that go into achieving desired (and undesired) results through the Coordinated Entry system. This data element is intended to standardize data collection on core components of Coordinated Entry like access, assessment, referral, and prioritization.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/common-program-specific-data-elements/419-coordinated-entry-assessment/</t>
+  </si>
+  <si>
+    <t>The CE Assessment element is a flexible data element that collects an assessment date, location, and result. It allows CoCs to define their own assessment questions and responses and categorizes each assessment into different types: Crisis Needs or Housing Needs. This data element is intended to standardize data collection on core components of Coordinated Entry like access, assessment, referral, and prioritization.</t>
+  </si>
+  <si>
+    <t>To determine each bed-night utilized by a client in a Night-by-Night (NbN) shelter.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/common-program-specific-data-elements/414-bed-night-date/</t>
+  </si>
+  <si>
+    <t>To record the date the client became 'engaged' in project services after one or more contacts with a street outreach project or Night-by-Night shelter.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/common-program-specific-data-elements/413-date-of-engagement/</t>
+  </si>
+  <si>
+    <t>To record each contact with people experiencing homelessness by street outreach and other projects. This element provides information on the number of contacts required to engage the client as well as to document a current living situation each time the client is contacted.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/common-program-specific-data-elements/412-current-living-situation/</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/common-program-specific-data-elements/411-domestic-violence/</t>
+  </si>
+  <si>
+    <t>To indicate whether the Head of Household and other adults served are survivors of domestic violence. Ascertaining whether a person is a survivor of or fleeing from domestic violence is necessary to provide the person with the appropriate services to prevent further abuse and to treat the physical and psychological injuries from prior abuse. Also, ascertaining that a person may be experiencing domestic violence may be important for the safety of project staff and other clients. At the aggregate level, knowing the size of the population of persons experiencing homelessness who have also experienced domestic violence is critical for determining the resources needed to address the problem.</t>
+  </si>
+  <si>
+    <t>To indicate whether clients have a substance use disorder which contributes to their experience of homelessness or may be a factor in housing.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/common-program-specific-data-elements/410-substance-use-disorder/</t>
+  </si>
+  <si>
+    <t>To indicate whether clients have any mental health disorders which contribute to their experience of homelessness or may be a factor in housing.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/common-program-specific-data-elements/409-mental-health-disorder/</t>
+  </si>
+  <si>
+    <t>To indicate whether clients have HIV/AIDS which contributes to their experience of homelessness or may be a factor in housing.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/common-program-specific-data-elements/408-hivaids/</t>
+  </si>
+  <si>
+    <t>To indicate whether clients have any disabling special needs which contribute to their experience of homelessness or may be a factor in housing.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/common-program-specific-data-elements/407-chronic-health-condition/</t>
+  </si>
+  <si>
+    <t>To indicate whether clients have a developmental disability which contributes to their experience of homelessness or may be a factor in housing.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/common-program-specific-data-elements/406-developmental-disability/</t>
+  </si>
+  <si>
+    <t>To indicate whether clients have a physical disability which contribute to their experience of homelessness or may be a factor in housing.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/common-program-specific-data-elements/405-physical-disability/</t>
+  </si>
+  <si>
+    <t>To determine whether clients are accessing all mainstream medical assistance benefits for which they may be eligible, and to ascertain a more complete picture of changes to economic circumstances between project start and exit.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/common-program-specific-data-elements/404-health-insurance/</t>
+  </si>
+  <si>
+    <t>To determine whether households are accessing all mainstream program benefits for which they are eligible at the time of project start and to allow for analyzing changes in the composition of non-cash benefits between project start and exit.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/common-program-specific-data-elements/403-non-cash-benefits/</t>
+  </si>
+  <si>
+    <t>To determine whether households are accessing all income sources for which they are eligible at the time of project start and to allow for analyzing changes in income between project start, annual assessment, and exit.
+Increase in income is a key performance measure of most federal partner programs. Collecting income information throughout a project stay supports plans to link clients with all income sources and benefits for which they are eligible and helps CoCs improve system design and partnerships by analyzing cross-systems connections to ensure access to additional income sources.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/common-program-specific-data-elements/402-income-and-sources/</t>
+  </si>
+  <si>
+    <t>To understand the type of moving on assistance provided to PSH participants.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/coc/c2-moving-on-assistance-provided/</t>
+  </si>
+  <si>
+    <t>To determine whether youth Heads of Household are accessing educational programs at the time of project start and exit, and to allow for analyzing changes in education status of youth between project start and exit.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/coc/c3-youth-education-status/</t>
+  </si>
+  <si>
+    <t>To measure the extent to which housing impacts participation in care for persons with HIV/AIDS in households served by all HOPWA component types.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/hopwa/w6-prescribed-anti-retroviral/</t>
+  </si>
+  <si>
+    <t>To determine whether clients exiting all HOPWA component types have remained stably housed.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/hopwa/w5-housing-assessment-at-exit/</t>
+  </si>
+  <si>
+    <t>To measure the extent to which housing impacts the health of persons with HIV/AIDS in households served by all HOPWA component types.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/hopwa/w4-t-cell-cd4-and-viral-load/</t>
+  </si>
+  <si>
+    <r>
+      <t>Medical assistance information is important to determine whether HIV positive clients in households served by all HOPWA component types are accessing medical assistance benefits for which they may be eligible. </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF333333"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Medical Assistance</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF333333"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> (W3) is designed to collect information on assistance provided to clients with HIV/AIDS.</t>
+    </r>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/hopwa/w3-medical-assistance/</t>
+  </si>
+  <si>
+    <t>To track HOPWA financial assistance provided to clients in Permanent Housing Placement, Tenant-Based Rental Assistance (TBRA) or Short-Term Rent, Mortgage, and Utilities (STRMU) during project participation.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/hopwa/w2-financial-assistance-hopwa/</t>
+  </si>
+  <si>
+    <t>To determine the services provided to clients during project participation.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/hopwa/w1-services-provided-hopwa/</t>
+  </si>
+  <si>
+    <t>Connection with SOAR is intended to determine if the client has been connected to the SSI/SSDI Outreach, Access, and Recovery (SOAR) program, regardless of whether that connection was established by the PATH provider or not.</t>
+  </si>
+  <si>
+    <t>HMIS Data Standards: PATH: P4 Connection with SOAR - HUD Exchange</t>
+  </si>
+  <si>
+    <t>To determine whether a client is eligible for the PATH program.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/path/p3-path-status/</t>
+  </si>
+  <si>
+    <t>To determine the referrals that are made on behalf of a client during project enrollment.</t>
+  </si>
+  <si>
+    <t>HMIS Data Standards: PATH: P2 Referrals Provided - HUD Exchange</t>
+  </si>
+  <si>
+    <t>To determine the PATH-funded services that are provided to a client during and throughout project enrollment and prior to project exit.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/path/p1-services-provided-path-funded/</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/va/v10-mental-health-consultation/</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/va/v9-hud-vash-exit-information/</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/va/v8-hud-vash-voucher-tracking/</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/va/v7-hp-targeting-criteria/</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/va/v6-vamc-station-number/</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/va/v4-percent-of-ami-ssvf-eligibility/</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/va/v3-financial-assistance-ssvf/</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/va/v2-services-provided-ssvf/</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/va/v1-veterans-information/</t>
+  </si>
+  <si>
+    <t>The purpose is to identify the extent of aftercare plans which were executed post-exit from the project.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/rhy/r20-aftercare-plans/</t>
+  </si>
+  <si>
+    <t>The purpose of this element is to determine the number of youth who exited to safe and appropriate destinations as determined by the youth (Head of Household and adult) themselves and as determined by the project/caseworker.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/rhy/r19-safe-and-appropriate-exit/</t>
+  </si>
+  <si>
+    <t>The purpose of this element is to identify the type and amount of counseling received by adults and Heads of Household enrolled in RHY projects.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/rhy/r18-counseling/</t>
+  </si>
+  <si>
+    <t>The purpose is to identify whether the youth completed the project or exited without completion. This data is only collected on heads of household and adults at project exit.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/rhy/r17-project-completion-status/</t>
+  </si>
+  <si>
+    <t>The purpose is to assess the extent of labor exploitation among youth experiencing homelessness.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/rhy/r16-labor-exploitationtrafficking/</t>
+  </si>
+  <si>
+    <t>The purpose is to assess the extent of sexual exploitation among youth experiencing homelessness.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/rhy/r15-commercial-sexual-exploitationsex-trafficking/</t>
+  </si>
+  <si>
+    <t>The RHY service connections enable projects to report on the services that they either directly provided to youth through their project or at their organization or which they facilitated being provided by another provider during the project stay for all Heads of Household and adults.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/rhy/r14-rhy-service-connections/</t>
+  </si>
+  <si>
+    <t>The purpose is to identify specific family issues faced by youth in RHY programs that may have contributed to the youth’s homelessness or is a factor in family reunification.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/rhy/r13-family-critical-issues/</t>
+  </si>
+  <si>
+    <t>The purpose is to identify clients with juvenile justice system history.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/rhy/r12-formerly-a-ward-of-juvenile-justice-system/</t>
+  </si>
+  <si>
+    <t>The purpose is to identify clients with child welfare or foster care histories.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/rhy/r11-formerly-a-ward-of-child-welfarefoster-care-agency/</t>
+  </si>
+  <si>
+    <t>The purpose is to determine the number of people starting projects while pregnant and to determine eligibility for benefits and need for services.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/rhy/r10-pregnancy-status/</t>
+  </si>
+  <si>
+    <t>Information on health status (general health, dental health, and mental health) is a first step to identifying what types of health services a client may need. This element permits comparison between homeless youth to other youth their age as well as measure a change in status from project start to project exit for all Heads of Household and adults.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/rhy/r9-mental-health-status/</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/rhy/r8-dental-health-status/</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/rhy/r7-general-health-status/</t>
+  </si>
+  <si>
+    <t>The purpose is to assess a client’s employment status and need for employment services as well as, when appropriate, measure a change in employment from project start to project exit for all Heads of Household and adults.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/rhy/r6-employment-status/</t>
+  </si>
+  <si>
+    <t>The purpose is to identify the educational status of youth served in RHY projects as well as, when appropriate, measure a change in school status from project start to project exit for all Heads of Household and youth.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/rhy/r5-school-status/</t>
+  </si>
+  <si>
+    <t>The purpose is to identify the educational attainment of youth served in RHY projects as well as, when appropriate, measure a change in education from project start to project exit for all Heads of Household and youth.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/rhy/r4-last-grade-completed/</t>
+  </si>
+  <si>
+    <t>This element serves a three-fold purpose:
+Enables a BCP emergency shelter to record a youth that is not eligible under the FYSB-RHY program and collect information about them. Upon reporting to RHY for the federal transfer, RHY is then able to remove these youth from their program and congressional reports.
+Facilitates the local CoC and HMIS to utilize participation in BCP as part of their point-in-time and other counts and measures.
+Identifies the number of runaway youth.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/rhy/r2-rhy-bcp-status/</t>
+  </si>
+  <si>
+    <t>Referral sources indicate the person, place or organization that referred the youth to the project they are entering.</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/rhy/r1-referral-source/</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/metadata-elements/501-date-created/</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/metadata-elements/502-date-updated/</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/metadata-elements/503-data-collection-stage/</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/metadata-elements/504-information-date/</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/metadata-elements/505-project-identifier/</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/metadata-elements/506-enrollment-identifier/</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/metadata-elements/507-user-identifier/</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/metadata-elements/508-personal-identifier/</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/metadata-elements/509-household-identifier/</t>
+  </si>
+  <si>
+    <t>https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/metadata-elements/510-implementation-identifier/</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1369,6 +1938,27 @@
       <sz val="11"/>
       <color rgb="FF008000"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF333333"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF333333"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1398,10 +1988,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1412,8 +2003,14 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1480,13 +2077,67 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1457325</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>552450</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="AutoShape 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{36B08963-A50F-519A-1EC9-09B9ABB3EC3F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="9525000" cy="9525000"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="HMISDataElements" displayName="HMISDataElements" ref="A1:I88">
-  <autoFilter ref="A1:I88" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="HMISDataElements" displayName="HMISDataElements" ref="A1:K88">
+  <autoFilter ref="A1:K88" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Element Identifier"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Element Name"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Element Type"/>
@@ -1496,6 +2147,8 @@
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Collection Point"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="System Logic and Other System Issues"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="CSV"/>
+    <tableColumn id="10" xr3:uid="{9E84F1CA-4630-477B-8C60-24667C78AF32}" name="Rationale"/>
+    <tableColumn id="11" xr3:uid="{5E922C16-42DF-4F25-8355-EE887AB63D4B}" name="Data Collection Instruction"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1677,21 +2330,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I88"/>
+  <dimension ref="A1:K88"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="38" customWidth="1"/>
-    <col min="3" max="3" width="20" customWidth="1"/>
-    <col min="4" max="4" width="45" customWidth="1"/>
-    <col min="5" max="5" width="38" customWidth="1"/>
-    <col min="6" max="6" width="28" customWidth="1"/>
-    <col min="7" max="7" width="40" customWidth="1"/>
-    <col min="8" max="8" width="90" customWidth="1"/>
-    <col min="9" max="9" width="24" customWidth="1"/>
+    <col min="3" max="3" width="20" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="45" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="38" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="28" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="40" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="90" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="24" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="27.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1719,8 +2374,14 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="J1" t="s">
+        <v>391</v>
+      </c>
+      <c r="K1" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
@@ -1748,8 +2409,14 @@
       <c r="I2" s="2" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="J2" s="4" t="s">
+        <v>393</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>18</v>
       </c>
@@ -1777,8 +2444,14 @@
       <c r="I3" s="3" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="J3" t="s">
+        <v>394</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>23</v>
       </c>
@@ -1806,8 +2479,14 @@
       <c r="I4" s="2" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="J4" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>28</v>
       </c>
@@ -1835,8 +2514,14 @@
       <c r="I5" s="3" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" ht="120" x14ac:dyDescent="0.25">
+      <c r="J5" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="120" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>32</v>
       </c>
@@ -1864,8 +2549,14 @@
       <c r="I6" s="2" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="J6" s="4" t="s">
+        <v>397</v>
+      </c>
+      <c r="K6" s="6" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>39</v>
       </c>
@@ -1893,8 +2584,14 @@
       <c r="I7" s="3" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="J7" s="4" t="s">
+        <v>398</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>45</v>
       </c>
@@ -1922,8 +2619,14 @@
       <c r="I8" s="2" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J8" s="4" t="s">
+        <v>399</v>
+      </c>
+      <c r="K8" s="6" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>50</v>
       </c>
@@ -1951,8 +2654,14 @@
       <c r="I9" s="3" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J9" s="4" t="s">
+        <v>407</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>57</v>
       </c>
@@ -1980,8 +2689,14 @@
       <c r="I10" s="2" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J10" s="5" t="s">
+        <v>409</v>
+      </c>
+      <c r="K10" s="6" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>60</v>
       </c>
@@ -2009,8 +2724,14 @@
       <c r="I11" s="3" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J11" s="4" t="s">
+        <v>411</v>
+      </c>
+      <c r="K11" s="6" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>63</v>
       </c>
@@ -2038,8 +2759,14 @@
       <c r="I12" s="2" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J12" s="4" t="s">
+        <v>413</v>
+      </c>
+      <c r="K12" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>66</v>
       </c>
@@ -2067,8 +2794,14 @@
       <c r="I13" s="3" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="14" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="J13" s="4" t="s">
+        <v>415</v>
+      </c>
+      <c r="K13" s="6" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>70</v>
       </c>
@@ -2096,8 +2829,14 @@
       <c r="I14" s="2" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J14" s="4" t="s">
+        <v>419</v>
+      </c>
+      <c r="K14" s="6" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>75</v>
       </c>
@@ -2125,8 +2864,14 @@
       <c r="I15" s="3" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J15" s="4" t="s">
+        <v>420</v>
+      </c>
+      <c r="K15" s="6" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>79</v>
       </c>
@@ -2154,8 +2899,14 @@
       <c r="I16" s="2" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J16" s="4" t="s">
+        <v>423</v>
+      </c>
+      <c r="K16" s="6" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>84</v>
       </c>
@@ -2183,8 +2934,14 @@
       <c r="I17" s="3" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J17" s="4" t="s">
+        <v>425</v>
+      </c>
+      <c r="K17" s="6" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>87</v>
       </c>
@@ -2212,8 +2969,14 @@
       <c r="I18" s="2" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J18" s="4" t="s">
+        <v>426</v>
+      </c>
+      <c r="K18" s="6" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>90</v>
       </c>
@@ -2241,8 +3004,14 @@
       <c r="I19" s="3" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="20" spans="1:9" ht="135" x14ac:dyDescent="0.25">
+      <c r="J19" s="4" t="s">
+        <v>428</v>
+      </c>
+      <c r="K19" s="6" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="135" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>94</v>
       </c>
@@ -2270,8 +3039,14 @@
       <c r="I20" s="2" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="21" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="J20" s="4" t="s">
+        <v>429</v>
+      </c>
+      <c r="K20" s="6" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>100</v>
       </c>
@@ -2299,8 +3074,14 @@
       <c r="I21" s="3" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="22" spans="1:9" ht="120" x14ac:dyDescent="0.25">
+      <c r="J21" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="K21" s="6" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="120" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>107</v>
       </c>
@@ -2328,8 +3109,14 @@
       <c r="I22" s="2" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="23" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="J22" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="K22" s="6" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>111</v>
       </c>
@@ -2357,8 +3144,14 @@
       <c r="I23" s="3" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="24" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="J23" s="5" t="s">
+        <v>463</v>
+      </c>
+      <c r="K23" s="6" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>118</v>
       </c>
@@ -2386,8 +3179,14 @@
       <c r="I24" s="2" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="25" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="J24" s="4" t="s">
+        <v>461</v>
+      </c>
+      <c r="K24" s="6" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>120</v>
       </c>
@@ -2415,8 +3214,14 @@
       <c r="I25" s="3" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="26" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="J25" s="4" t="s">
+        <v>459</v>
+      </c>
+      <c r="K25" s="6" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>123</v>
       </c>
@@ -2444,8 +3249,14 @@
       <c r="I26" s="2" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="27" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="J26" s="4" t="s">
+        <v>457</v>
+      </c>
+      <c r="K26" s="6" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>127</v>
       </c>
@@ -2473,8 +3284,14 @@
       <c r="I27" s="3" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="28" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="J27" s="4" t="s">
+        <v>455</v>
+      </c>
+      <c r="K27" s="6" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>129</v>
       </c>
@@ -2502,8 +3319,14 @@
       <c r="I28" s="2" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="29" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="J28" s="4" t="s">
+        <v>453</v>
+      </c>
+      <c r="K28" s="6" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>132</v>
       </c>
@@ -2531,8 +3354,14 @@
       <c r="I29" s="3" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="30" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="J29" s="4" t="s">
+        <v>451</v>
+      </c>
+      <c r="K29" s="6" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>134</v>
       </c>
@@ -2560,8 +3389,14 @@
       <c r="I30" s="2" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="31" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="J30" s="4" t="s">
+        <v>449</v>
+      </c>
+      <c r="K30" s="6" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>136</v>
       </c>
@@ -2589,8 +3424,14 @@
       <c r="I31" s="3" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="32" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="J31" s="4" t="s">
+        <v>447</v>
+      </c>
+      <c r="K31" s="6" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>139</v>
       </c>
@@ -2618,8 +3459,14 @@
       <c r="I32" s="2" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="33" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+      <c r="J32" s="4" t="s">
+        <v>446</v>
+      </c>
+      <c r="K32" s="6" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
         <v>144</v>
       </c>
@@ -2647,8 +3494,14 @@
       <c r="I33" s="3" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="34" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="J33" s="4" t="s">
+        <v>443</v>
+      </c>
+      <c r="K33" s="6" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>151</v>
       </c>
@@ -2676,8 +3529,14 @@
       <c r="I34" s="2" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="35" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="J34" s="4" t="s">
+        <v>441</v>
+      </c>
+      <c r="K34" s="6" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
         <v>157</v>
       </c>
@@ -2705,8 +3564,14 @@
       <c r="I35" s="3" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="36" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="J35" t="s">
+        <v>439</v>
+      </c>
+      <c r="K35" s="6" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>164</v>
       </c>
@@ -2734,8 +3599,14 @@
       <c r="I36" s="2" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="37" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="J36" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="K36" s="6" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
         <v>171</v>
       </c>
@@ -2763,8 +3634,14 @@
       <c r="I37" s="3" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="38" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="J37" s="4" t="s">
+        <v>436</v>
+      </c>
+      <c r="K37" s="6" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>175</v>
       </c>
@@ -2792,8 +3669,14 @@
       <c r="I38" s="2" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="39" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="J38" s="4" t="s">
+        <v>434</v>
+      </c>
+      <c r="K38" s="6" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
         <v>179</v>
       </c>
@@ -2821,8 +3704,14 @@
       <c r="I39" s="3" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="40" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="J39" s="4" t="s">
+        <v>465</v>
+      </c>
+      <c r="K39" s="6" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>185</v>
       </c>
@@ -2850,8 +3739,14 @@
       <c r="I40" s="2" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="41" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+      <c r="J40" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="K40" s="6" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
         <v>192</v>
       </c>
@@ -2879,8 +3774,14 @@
       <c r="I41" s="3" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="42" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="J41" s="4" t="s">
+        <v>479</v>
+      </c>
+      <c r="K41" s="6" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>198</v>
       </c>
@@ -2908,8 +3809,14 @@
       <c r="I42" s="2" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="43" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+      <c r="J42" s="4" t="s">
+        <v>477</v>
+      </c>
+      <c r="K42" s="6" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
         <v>202</v>
       </c>
@@ -2937,8 +3844,14 @@
       <c r="I43" s="3" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="44" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+      <c r="J43" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="K43" s="6" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>206</v>
       </c>
@@ -2966,8 +3879,14 @@
       <c r="I44" s="2" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="45" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+      <c r="J44" s="4" t="s">
+        <v>473</v>
+      </c>
+      <c r="K44" s="6" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
         <v>209</v>
       </c>
@@ -2995,8 +3914,14 @@
       <c r="I45" s="3" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="46" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+      <c r="J45" s="4" t="s">
+        <v>471</v>
+      </c>
+      <c r="K45" s="6" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>213</v>
       </c>
@@ -3024,8 +3949,14 @@
       <c r="I46" s="2" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="47" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="J46" s="4" t="s">
+        <v>469</v>
+      </c>
+      <c r="K46" s="6" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
         <v>217</v>
       </c>
@@ -3053,8 +3984,14 @@
       <c r="I47" s="3" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="48" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="J47" s="4" t="s">
+        <v>487</v>
+      </c>
+      <c r="K47" s="6" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>221</v>
       </c>
@@ -3082,8 +4019,14 @@
       <c r="I48" s="2" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="49" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="J48" s="4" t="s">
+        <v>485</v>
+      </c>
+      <c r="K48" s="6" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
         <v>224</v>
       </c>
@@ -3111,8 +4054,14 @@
       <c r="I49" s="3" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="50" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="J49" s="4" t="s">
+        <v>483</v>
+      </c>
+      <c r="K49" s="6" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>228</v>
       </c>
@@ -3140,8 +4089,14 @@
       <c r="I50" s="2" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="51" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="J50" s="4" t="s">
+        <v>481</v>
+      </c>
+      <c r="K50" s="6" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
         <v>232</v>
       </c>
@@ -3169,8 +4124,14 @@
       <c r="I51" s="3" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="52" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="J51" s="4" t="s">
+        <v>532</v>
+      </c>
+      <c r="K51" s="6" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>237</v>
       </c>
@@ -3198,8 +4159,14 @@
       <c r="I52" s="2" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="53" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+      <c r="J52" s="5" t="s">
+        <v>530</v>
+      </c>
+      <c r="K52" s="6" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
         <v>242</v>
       </c>
@@ -3227,8 +4194,14 @@
       <c r="I53" s="3" t="s">
         <v>247</v>
       </c>
-    </row>
-    <row r="54" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="J53" s="4" t="s">
+        <v>528</v>
+      </c>
+      <c r="K53" s="6" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>248</v>
       </c>
@@ -3256,8 +4229,14 @@
       <c r="I54" s="2" t="s">
         <v>247</v>
       </c>
-    </row>
-    <row r="55" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="J54" t="s">
+        <v>526</v>
+      </c>
+      <c r="K54" s="6" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
         <v>250</v>
       </c>
@@ -3285,8 +4264,14 @@
       <c r="I55" s="3" t="s">
         <v>247</v>
       </c>
-    </row>
-    <row r="56" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="J55" s="4" t="s">
+        <v>524</v>
+      </c>
+      <c r="K55" s="6" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>254</v>
       </c>
@@ -3314,8 +4299,14 @@
       <c r="I56" s="2" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="57" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="J56" s="4" t="s">
+        <v>520</v>
+      </c>
+      <c r="K56" s="6" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
         <v>257</v>
       </c>
@@ -3343,8 +4334,14 @@
       <c r="I57" s="3" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="58" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="J57" s="4" t="s">
+        <v>520</v>
+      </c>
+      <c r="K57" s="6" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
         <v>260</v>
       </c>
@@ -3372,8 +4369,14 @@
       <c r="I58" s="2" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="59" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="J58" s="4" t="s">
+        <v>520</v>
+      </c>
+      <c r="K58" s="6" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A59" s="3" t="s">
         <v>262</v>
       </c>
@@ -3401,8 +4404,14 @@
       <c r="I59" s="3" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="60" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="J59" t="s">
+        <v>518</v>
+      </c>
+      <c r="K59" s="6" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
         <v>267</v>
       </c>
@@ -3430,8 +4439,14 @@
       <c r="I60" s="2" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="61" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="J60" s="4" t="s">
+        <v>516</v>
+      </c>
+      <c r="K60" s="6" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="s">
         <v>269</v>
       </c>
@@ -3459,8 +4474,14 @@
       <c r="I61" s="3" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="62" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="J61" t="s">
+        <v>514</v>
+      </c>
+      <c r="K61" s="6" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
         <v>271</v>
       </c>
@@ -3488,8 +4509,14 @@
       <c r="I62" s="2" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="63" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="J62" s="4" t="s">
+        <v>512</v>
+      </c>
+      <c r="K62" s="6" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A63" s="3" t="s">
         <v>273</v>
       </c>
@@ -3517,8 +4544,14 @@
       <c r="I63" s="3" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="64" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+      <c r="J63" t="s">
+        <v>510</v>
+      </c>
+      <c r="K63" s="6" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
         <v>279</v>
       </c>
@@ -3546,8 +4579,14 @@
       <c r="I64" s="2" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="65" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="J64" s="4" t="s">
+        <v>508</v>
+      </c>
+      <c r="K64" s="6" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
         <v>282</v>
       </c>
@@ -3575,8 +4614,14 @@
       <c r="I65" s="3" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="66" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="J65" s="4" t="s">
+        <v>506</v>
+      </c>
+      <c r="K65" s="6" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
         <v>286</v>
       </c>
@@ -3604,8 +4649,14 @@
       <c r="I66" s="2" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="67" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="J66" s="4" t="s">
+        <v>504</v>
+      </c>
+      <c r="K66" s="6" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A67" s="3" t="s">
         <v>290</v>
       </c>
@@ -3633,8 +4684,14 @@
       <c r="I67" s="3" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="68" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="J67" s="4" t="s">
+        <v>502</v>
+      </c>
+      <c r="K67" s="6" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
         <v>292</v>
       </c>
@@ -3662,8 +4719,14 @@
       <c r="I68" s="2" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="69" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="J68" s="4" t="s">
+        <v>500</v>
+      </c>
+      <c r="K68" s="6" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A69" s="3" t="s">
         <v>295</v>
       </c>
@@ -3691,8 +4754,14 @@
       <c r="I69" s="3" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="70" spans="1:9" ht="105" x14ac:dyDescent="0.25">
+      <c r="J69" s="4" t="s">
+        <v>498</v>
+      </c>
+      <c r="K69" s="6" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" ht="105" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
         <v>299</v>
       </c>
@@ -3720,8 +4789,11 @@
       <c r="I70" s="2" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="71" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="K70" s="6" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A71" s="3" t="s">
         <v>305</v>
       </c>
@@ -3749,8 +4821,11 @@
       <c r="I71" s="3" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="72" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="K71" s="6" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
         <v>311</v>
       </c>
@@ -3778,8 +4853,11 @@
       <c r="I72" s="2" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="73" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="K72" s="6" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A73" s="3" t="s">
         <v>315</v>
       </c>
@@ -3807,8 +4885,11 @@
       <c r="I73" s="3" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="74" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="K73" s="6" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
         <v>318</v>
       </c>
@@ -3836,8 +4917,11 @@
       <c r="I74" s="2" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="75" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="K74" s="6" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A75" s="3" t="s">
         <v>322</v>
       </c>
@@ -3865,8 +4949,11 @@
       <c r="I75" s="3" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="76" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="K75" s="6" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
         <v>327</v>
       </c>
@@ -3894,8 +4981,11 @@
       <c r="I76" s="2" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="77" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="K76" s="6" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A77" s="3" t="s">
         <v>331</v>
       </c>
@@ -3923,8 +5013,11 @@
       <c r="I77" s="3" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="78" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="K77" s="6" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
         <v>333</v>
       </c>
@@ -3952,8 +5045,11 @@
       <c r="I78" s="2" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="79" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="K78" s="6" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A79" s="3" t="s">
         <v>338</v>
       </c>
@@ -3981,8 +5077,11 @@
       <c r="I79" s="3" t="s">
         <v>343</v>
       </c>
-    </row>
-    <row r="80" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="K79" s="6" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
         <v>344</v>
       </c>
@@ -4010,8 +5109,11 @@
       <c r="I80" s="2" t="s">
         <v>349</v>
       </c>
-    </row>
-    <row r="81" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="K80" s="6" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="s">
         <v>350</v>
       </c>
@@ -4039,8 +5141,11 @@
       <c r="I81" s="3" t="s">
         <v>355</v>
       </c>
-    </row>
-    <row r="82" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="K81" s="6" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
         <v>356</v>
       </c>
@@ -4068,8 +5173,11 @@
       <c r="I82" s="2" t="s">
         <v>361</v>
       </c>
-    </row>
-    <row r="83" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="K82" s="6" t="s">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A83" s="3" t="s">
         <v>362</v>
       </c>
@@ -4097,8 +5205,11 @@
       <c r="I83" s="3" t="s">
         <v>367</v>
       </c>
-    </row>
-    <row r="84" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="K83" s="6" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
         <v>368</v>
       </c>
@@ -4126,8 +5237,11 @@
       <c r="I84" s="2" t="s">
         <v>372</v>
       </c>
-    </row>
-    <row r="85" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="K84" s="6" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="85" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A85" s="3" t="s">
         <v>373</v>
       </c>
@@ -4155,8 +5269,11 @@
       <c r="I85" s="3" t="s">
         <v>377</v>
       </c>
-    </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K85" s="6" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
         <v>378</v>
       </c>
@@ -4184,8 +5301,11 @@
       <c r="I86" s="2" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K86" s="6" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A87" s="3" t="s">
         <v>381</v>
       </c>
@@ -4213,8 +5333,11 @@
       <c r="I87" s="3" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K87" s="6" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
         <v>384</v>
       </c>
@@ -4242,13 +5365,97 @@
       <c r="I88" s="2" t="s">
         <v>390</v>
       </c>
+      <c r="K88" s="6" t="s">
+        <v>543</v>
+      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="K8" r:id="rId1" xr:uid="{8B77E5CA-F975-4728-AAB2-36DAB86E0DE5}"/>
+    <hyperlink ref="K10" r:id="rId2" xr:uid="{28E2F27F-C8FE-4E09-ACD8-04D212CBCDEC}"/>
+    <hyperlink ref="K11" r:id="rId3" xr:uid="{FD9D3FF1-7E66-4121-ABDE-48941917B844}"/>
+    <hyperlink ref="K13" r:id="rId4" xr:uid="{DEC60A77-7EEE-4019-B63C-3B1998428E83}"/>
+    <hyperlink ref="K14" r:id="rId5" xr:uid="{C8446DCC-1FE7-4AD9-A55E-EF5BF6A35260}"/>
+    <hyperlink ref="K15" r:id="rId6" xr:uid="{9A604731-F7A1-4674-9436-00702D1AD271}"/>
+    <hyperlink ref="K16" r:id="rId7" xr:uid="{42049C99-ACE7-4860-B3E2-4A6C83AF64FF}"/>
+    <hyperlink ref="K17" r:id="rId8" xr:uid="{4E002A20-99B5-44D6-9E23-B8CA52008A51}"/>
+    <hyperlink ref="K18" r:id="rId9" xr:uid="{0301C95A-8738-4DD8-81B7-92A8E2669B18}"/>
+    <hyperlink ref="K19" r:id="rId10" xr:uid="{72961C90-4F1C-4ADB-91A3-393D8F088273}"/>
+    <hyperlink ref="K20" r:id="rId11" xr:uid="{9F09D46F-B4E4-4628-932D-67D4B8B9945D}"/>
+    <hyperlink ref="K21" r:id="rId12" xr:uid="{569F39E8-5320-40EC-8780-F0009C445177}"/>
+    <hyperlink ref="K22" r:id="rId13" xr:uid="{B7E517BE-B063-4F69-93A1-C099208A537D}"/>
+    <hyperlink ref="K38" r:id="rId14" xr:uid="{3E3869D4-CAD3-4C5B-884C-702B2A2E7110}"/>
+    <hyperlink ref="K37" r:id="rId15" xr:uid="{32A52877-B84A-4F73-829E-A019AC633567}"/>
+    <hyperlink ref="K36" r:id="rId16" xr:uid="{DEC268D9-919A-44DF-B88D-1CD2BF36697C}"/>
+    <hyperlink ref="K35" r:id="rId17" xr:uid="{8CF9CEC9-E1CB-4096-8434-49448B79EA5A}"/>
+    <hyperlink ref="K34" r:id="rId18" xr:uid="{92E4DEBB-58AD-462B-8DE8-8517624C55A4}"/>
+    <hyperlink ref="K33" r:id="rId19" xr:uid="{93AAF44B-66A5-46C4-8613-3CBFA18738F9}"/>
+    <hyperlink ref="K32" r:id="rId20" xr:uid="{25E71BE2-7A64-4466-968B-7C60F2582E60}"/>
+    <hyperlink ref="K31" r:id="rId21" xr:uid="{4529E3E0-4BD4-43E3-B847-04D3AB61A426}"/>
+    <hyperlink ref="K30" r:id="rId22" xr:uid="{29641A77-D543-4627-BAD1-FF43285E9ADB}"/>
+    <hyperlink ref="K29" r:id="rId23" xr:uid="{85FD9845-08FF-4D10-9D47-82F36019097F}"/>
+    <hyperlink ref="K28" r:id="rId24" xr:uid="{4037F8D4-1137-4219-AF94-4E9CF0C0DF35}"/>
+    <hyperlink ref="K27" r:id="rId25" xr:uid="{F9AD3ADE-D9F6-46B6-B22A-4F81EB28018F}"/>
+    <hyperlink ref="K26" r:id="rId26" xr:uid="{2A2CDFAE-F40C-42D2-A905-BA3B25579E1E}"/>
+    <hyperlink ref="K25" r:id="rId27" xr:uid="{37B44276-9025-4EDE-A5CA-9A25718E0C41}"/>
+    <hyperlink ref="K24" r:id="rId28" xr:uid="{15EAAA09-7E78-4906-B599-3C4CF0F1E292}"/>
+    <hyperlink ref="K23" r:id="rId29" xr:uid="{17AF2B3A-5253-41BF-A5BD-8323310BC860}"/>
+    <hyperlink ref="K39" r:id="rId30" xr:uid="{2A2C3F82-40AC-4CE7-839B-5C0F22D65FA5}"/>
+    <hyperlink ref="K40" r:id="rId31" xr:uid="{732FC84C-827B-40E1-B732-8241A726D436}"/>
+    <hyperlink ref="K46" r:id="rId32" xr:uid="{93F8D487-45CA-435D-B7E5-F165B60645E3}"/>
+    <hyperlink ref="K45" r:id="rId33" xr:uid="{F5FAEE9F-0B4C-4B3E-81D1-268E7075963A}"/>
+    <hyperlink ref="K44" r:id="rId34" xr:uid="{3F0B7D42-40B2-4F54-BD09-0CA0BB69AE05}"/>
+    <hyperlink ref="K43" r:id="rId35" xr:uid="{E53E1779-9CC0-4BDE-92F1-5966EC7A4BAA}"/>
+    <hyperlink ref="K42" r:id="rId36" xr:uid="{E5D4EDB8-8039-4AAA-ADF8-B15CAF0F13F5}"/>
+    <hyperlink ref="K41" r:id="rId37" xr:uid="{AB81F7E2-BB94-497A-AADB-02274827FA9F}"/>
+    <hyperlink ref="K50" r:id="rId38" display="https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/path/p4-connection-with-soar/" xr:uid="{B3CDDE6B-C299-48EC-8F49-2189BD8E1D42}"/>
+    <hyperlink ref="K49" r:id="rId39" xr:uid="{75084C80-23CE-4A30-8BAB-5D9CAD435FBD}"/>
+    <hyperlink ref="K48" r:id="rId40" display="https://www.hudexchange.info/programs/hmis/hmis-data-standards/standards/path/p2-referrals-provided-path/" xr:uid="{0713210A-2D41-4C3C-B779-23653B7757F5}"/>
+    <hyperlink ref="K47" r:id="rId41" xr:uid="{99564E44-8A2B-45B5-9A8C-AF2636485CE4}"/>
+    <hyperlink ref="K78" r:id="rId42" xr:uid="{0E078571-70C1-42DD-AD31-06B5BF2F04DC}"/>
+    <hyperlink ref="K77" r:id="rId43" xr:uid="{40E77B97-2EF9-4C34-B343-21B221F77B8C}"/>
+    <hyperlink ref="K76" r:id="rId44" xr:uid="{00576C75-E1A2-451B-865C-81AE0CF13A0E}"/>
+    <hyperlink ref="K75" r:id="rId45" xr:uid="{BE77CA45-094C-4F3F-8D36-7CD731C72BEA}"/>
+    <hyperlink ref="K74" r:id="rId46" xr:uid="{41C162D2-23F8-409C-84C5-A47E7550C9C3}"/>
+    <hyperlink ref="K73" r:id="rId47" xr:uid="{0E87C810-2B0E-49E3-8055-A942FE02CDF3}"/>
+    <hyperlink ref="K72" r:id="rId48" xr:uid="{D3F103D5-1B4D-483E-A3E5-8ADB4218682B}"/>
+    <hyperlink ref="K71" r:id="rId49" xr:uid="{BDD88B58-4700-488E-AC44-B46B566B1F0F}"/>
+    <hyperlink ref="K70" r:id="rId50" xr:uid="{13340F19-0F2F-40B3-A33F-200060A4B3E2}"/>
+    <hyperlink ref="K69" r:id="rId51" xr:uid="{39420B99-693A-4DA9-A246-B424985B0C17}"/>
+    <hyperlink ref="K68" r:id="rId52" xr:uid="{630425DD-E499-4722-8F24-77D5FF0E5C2C}"/>
+    <hyperlink ref="K67" r:id="rId53" xr:uid="{A1868627-086A-4BC6-9C1E-446C7225235E}"/>
+    <hyperlink ref="K66" r:id="rId54" xr:uid="{D6EC7B78-D5E6-41A4-AB13-928AED440D27}"/>
+    <hyperlink ref="K65" r:id="rId55" xr:uid="{8E4346B4-E2A7-40B8-B906-5409C8CD1736}"/>
+    <hyperlink ref="K64" r:id="rId56" xr:uid="{AF0BD171-7EA6-4915-85B9-61A400B1513A}"/>
+    <hyperlink ref="K63" r:id="rId57" xr:uid="{8D52977B-7D28-482F-8881-EB6091AE43D5}"/>
+    <hyperlink ref="K62" r:id="rId58" xr:uid="{37B4D8F9-DAEF-49FF-AF89-E06BF99FA888}"/>
+    <hyperlink ref="K61" r:id="rId59" xr:uid="{5DD50909-940F-4F58-A9D0-84D245447B61}"/>
+    <hyperlink ref="K60" r:id="rId60" xr:uid="{06552883-64E7-4FC5-A733-DB792E0CB804}"/>
+    <hyperlink ref="K59" r:id="rId61" xr:uid="{DFEE179C-F6D7-46AD-9DBD-DC018F43DB14}"/>
+    <hyperlink ref="K58" r:id="rId62" xr:uid="{92C54279-7108-4220-B098-E6511DC23A08}"/>
+    <hyperlink ref="K57" r:id="rId63" xr:uid="{AB9618DD-A716-4106-8AF2-70BCDE046C73}"/>
+    <hyperlink ref="K56" r:id="rId64" xr:uid="{91FB3067-4980-4ACD-A82F-3E11892FE287}"/>
+    <hyperlink ref="K55" r:id="rId65" xr:uid="{807EEF6D-1CE4-456B-9C82-C61C468A020B}"/>
+    <hyperlink ref="K54" r:id="rId66" xr:uid="{3CA9ABBC-F7BB-437B-A0D9-76E903601D1E}"/>
+    <hyperlink ref="K53" r:id="rId67" xr:uid="{C294093B-421F-495C-A82A-D41EC4DA7A7C}"/>
+    <hyperlink ref="K52" r:id="rId68" xr:uid="{56CC7AC9-B8B3-47AB-90E4-4A2CB578C847}"/>
+    <hyperlink ref="K51" r:id="rId69" xr:uid="{E9480240-D9F4-4662-A23F-7266AADFC662}"/>
+    <hyperlink ref="K79" r:id="rId70" xr:uid="{10134A0D-6312-40A2-8A56-F1B9B92547C0}"/>
+    <hyperlink ref="K80" r:id="rId71" xr:uid="{B635A48D-CA00-4651-BABA-B17FDF12A9B9}"/>
+    <hyperlink ref="K81" r:id="rId72" xr:uid="{5B982BB3-E433-471D-BF59-F982425CF607}"/>
+    <hyperlink ref="K82" r:id="rId73" xr:uid="{E6B163D7-EDD0-4D09-BB01-70186C5C5195}"/>
+    <hyperlink ref="K83" r:id="rId74" xr:uid="{C920A5DA-A386-4112-8F81-1C1A1C61AF5E}"/>
+    <hyperlink ref="K84" r:id="rId75" xr:uid="{33EA1123-9BE3-4F2E-8F5C-50C5FDB047FC}"/>
+    <hyperlink ref="K85" r:id="rId76" xr:uid="{D48A032C-C5C0-41E0-96B6-6389E2AB6653}"/>
+    <hyperlink ref="K86" r:id="rId77" xr:uid="{24366C9C-2B96-4C4F-B829-C6BE15EAA9B6}"/>
+    <hyperlink ref="K87" r:id="rId78" xr:uid="{5BD8A43C-4381-4331-9333-3CAAB7228F41}"/>
+    <hyperlink ref="K88" r:id="rId79" xr:uid="{1887BCA5-4F70-4EB3-8469-B992CE9098F0}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
+  <drawing r:id="rId80"/>
+  <legacyDrawing r:id="rId81"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId82"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>